<commit_message>
드릴 매니저 (DrillComponent) 구현
메인 씬 Drill 오브젝트에 컴포넌트로 들어가 있음.
</commit_message>
<xml_diff>
--- a/Assets/100_Data/XlsxFiles/Drill_Data.xlsx
+++ b/Assets/100_Data/XlsxFiles/Drill_Data.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Coding\Drill_Game\Assets\100_Data\XlsxFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\koseonghyeon\Desktop\Drill_Game\Drill_game\Assets\100_Data\XlsxFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2754A681-E3A4-42C6-93DA-FC6B7776E76B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13965" windowHeight="9705"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
   <si>
     <t>Id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -93,13 +94,21 @@
   </si>
   <si>
     <t>티타늄 드릴</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>stone_drill</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>copper_drill</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -161,14 +170,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="표1" displayName="표1" ref="A1:E8" totalsRowShown="0">
-  <autoFilter ref="A1:E8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="표1" displayName="표1" ref="A1:E8" totalsRowShown="0">
+  <autoFilter ref="A1:E8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="Id"/>
-    <tableColumn id="2" name="Name"/>
-    <tableColumn id="3" name="DisplayName"/>
-    <tableColumn id="5" name="Damage"/>
-    <tableColumn id="6" name="DrillSprite"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Name"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="DisplayName"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Damage"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="DrillSprite"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -436,7 +445,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -477,6 +486,9 @@
       <c r="D2">
         <v>1</v>
       </c>
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
@@ -491,6 +503,9 @@
       <c r="D3">
         <v>2</v>
       </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
@@ -505,6 +520,9 @@
       <c r="D4">
         <v>3</v>
       </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
@@ -519,6 +537,9 @@
       <c r="D5">
         <v>5</v>
       </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
@@ -533,6 +554,9 @@
       <c r="D6">
         <v>8</v>
       </c>
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
@@ -547,6 +571,9 @@
       <c r="D7">
         <v>13</v>
       </c>
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
@@ -560,6 +587,9 @@
       </c>
       <c r="D8">
         <v>21</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>